<commit_message>
main22,23 and 24th sep
</commit_message>
<xml_diff>
--- a/12604997.xlsx
+++ b/12604997.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45A98B2F-9ABD-4D3A-B082-852BD5781B4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD6F5D9-AD9B-48CA-90E6-FDC15A553E9C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="77">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -251,6 +251,21 @@
   </si>
   <si>
     <t>Not Good</t>
+  </si>
+  <si>
+    <t>Excellent</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Well</t>
+  </si>
+  <si>
+    <t>Little bit worry</t>
+  </si>
+  <si>
+    <t>try to make it great</t>
   </si>
 </sst>
 </file>
@@ -2272,70 +2287,142 @@
       </c>
     </row>
     <row r="33" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A33" s="13"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14"/>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="15" t="str">
+      <c r="A33" s="13">
+        <v>46287</v>
+      </c>
+      <c r="B33" s="14">
+        <v>565</v>
+      </c>
+      <c r="C33" s="14">
+        <v>25</v>
+      </c>
+      <c r="D33" s="14">
+        <v>120</v>
+      </c>
+      <c r="E33" s="14">
+        <v>45</v>
+      </c>
+      <c r="F33" s="14">
+        <v>300</v>
+      </c>
+      <c r="G33" s="14">
+        <v>6</v>
+      </c>
+      <c r="H33" s="14">
+        <v>25</v>
+      </c>
+      <c r="I33" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J33" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J33" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K33" s="16"/>
-      <c r="L33" s="16"/>
-      <c r="M33" s="16"/>
-      <c r="N33" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K33" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L33" s="16" t="s">
+        <v>73</v>
+      </c>
+      <c r="M33" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="N33" s="17" t="s">
+        <v>74</v>
+      </c>
     </row>
     <row r="34" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A34" s="13"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14"/>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14"/>
-      <c r="G34" s="14"/>
-      <c r="H34" s="14"/>
-      <c r="I34" s="15" t="str">
+      <c r="A34" s="13">
+        <v>46288</v>
+      </c>
+      <c r="B34" s="14">
+        <v>485</v>
+      </c>
+      <c r="C34" s="14">
+        <v>45</v>
+      </c>
+      <c r="D34" s="14">
+        <v>80</v>
+      </c>
+      <c r="E34" s="14">
+        <v>60</v>
+      </c>
+      <c r="F34" s="14">
+        <v>250</v>
+      </c>
+      <c r="G34" s="14">
+        <v>5</v>
+      </c>
+      <c r="H34" s="14">
+        <v>35</v>
+      </c>
+      <c r="I34" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J34" s="15" t="str">
+        <v>955</v>
+      </c>
+      <c r="J34" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K34" s="16"/>
-      <c r="L34" s="16"/>
-      <c r="M34" s="16"/>
-      <c r="N34" s="17"/>
+        <v>485</v>
+      </c>
+      <c r="K34" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L34" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="M34" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N34" s="17" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="35" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A35" s="13"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14"/>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14"/>
-      <c r="G35" s="14"/>
-      <c r="H35" s="14"/>
-      <c r="I35" s="15" t="str">
+      <c r="A35" s="13">
+        <v>46289</v>
+      </c>
+      <c r="B35" s="14">
+        <v>610</v>
+      </c>
+      <c r="C35" s="14">
+        <v>55</v>
+      </c>
+      <c r="D35" s="14">
+        <v>95</v>
+      </c>
+      <c r="E35" s="14">
+        <v>75</v>
+      </c>
+      <c r="F35" s="14">
+        <v>150</v>
+      </c>
+      <c r="G35" s="14">
+        <v>3</v>
+      </c>
+      <c r="H35" s="14">
+        <v>45</v>
+      </c>
+      <c r="I35" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J35" s="15" t="str">
+        <v>1030</v>
+      </c>
+      <c r="J35" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K35" s="16"/>
-      <c r="L35" s="16"/>
-      <c r="M35" s="16"/>
-      <c r="N35" s="17"/>
+        <v>410</v>
+      </c>
+      <c r="K35" s="16" t="s">
+        <v>72</v>
+      </c>
+      <c r="L35" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M35" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N35" s="17" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="36" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A36" s="13"/>

</xml_diff>

<commit_message>
main28 and 29 sept
</commit_message>
<xml_diff>
--- a/12604997.xlsx
+++ b/12604997.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB8CDFAA-A486-42F7-9234-72970DE625BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{37C5C061-3AF5-4333-B2AC-F336CECFF133}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="82">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -269,6 +269,18 @@
   </si>
   <si>
     <t>Good feeling better</t>
+  </si>
+  <si>
+    <t>feeling better</t>
+  </si>
+  <si>
+    <t>feeling great</t>
+  </si>
+  <si>
+    <t>ok good</t>
+  </si>
+  <si>
+    <t>trying to make day great</t>
   </si>
 </sst>
 </file>
@@ -2474,92 +2486,188 @@
       </c>
     </row>
     <row r="37" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A37" s="13"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14"/>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14"/>
-      <c r="G37" s="14"/>
-      <c r="H37" s="14"/>
-      <c r="I37" s="15" t="str">
+      <c r="A37" s="13">
+        <v>46291</v>
+      </c>
+      <c r="B37" s="14">
+        <v>565</v>
+      </c>
+      <c r="C37" s="14">
+        <v>25</v>
+      </c>
+      <c r="D37" s="14">
+        <v>85</v>
+      </c>
+      <c r="E37" s="14">
+        <v>75</v>
+      </c>
+      <c r="F37" s="14">
+        <v>150</v>
+      </c>
+      <c r="G37" s="14">
+        <v>0</v>
+      </c>
+      <c r="H37" s="14">
+        <v>25</v>
+      </c>
+      <c r="I37" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J37" s="15" t="str">
+        <v>925</v>
+      </c>
+      <c r="J37" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K37" s="16"/>
-      <c r="L37" s="16"/>
-      <c r="M37" s="16"/>
-      <c r="N37" s="17"/>
+        <v>515</v>
+      </c>
+      <c r="K37" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L37" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M37" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="N37" s="17" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="38" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A38" s="13"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14"/>
-      <c r="D38" s="14"/>
-      <c r="E38" s="14"/>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14"/>
-      <c r="I38" s="15" t="str">
+      <c r="A38" s="13">
+        <v>46292</v>
+      </c>
+      <c r="B38" s="14">
+        <v>660</v>
+      </c>
+      <c r="C38" s="14">
+        <v>35</v>
+      </c>
+      <c r="D38" s="14">
+        <v>125</v>
+      </c>
+      <c r="E38" s="14">
+        <v>120</v>
+      </c>
+      <c r="F38" s="14">
+        <v>0</v>
+      </c>
+      <c r="G38" s="14">
+        <v>0</v>
+      </c>
+      <c r="H38" s="14">
+        <v>35</v>
+      </c>
+      <c r="I38" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J38" s="15" t="str">
+        <v>975</v>
+      </c>
+      <c r="J38" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K38" s="16"/>
-      <c r="L38" s="16"/>
-      <c r="M38" s="16"/>
-      <c r="N38" s="17"/>
+        <v>465</v>
+      </c>
+      <c r="K38" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L38" s="16" t="s">
+        <v>65</v>
+      </c>
+      <c r="M38" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N38" s="17" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="39" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A39" s="13"/>
-      <c r="B39" s="14"/>
-      <c r="C39" s="14"/>
-      <c r="D39" s="14"/>
-      <c r="E39" s="14"/>
-      <c r="F39" s="14"/>
-      <c r="G39" s="14"/>
-      <c r="H39" s="14"/>
-      <c r="I39" s="15" t="str">
+      <c r="A39" s="13">
+        <v>46293</v>
+      </c>
+      <c r="B39" s="14">
+        <v>620</v>
+      </c>
+      <c r="C39" s="14">
+        <v>15</v>
+      </c>
+      <c r="D39" s="14">
+        <v>180</v>
+      </c>
+      <c r="E39" s="14">
+        <v>90</v>
+      </c>
+      <c r="F39" s="14">
+        <v>0</v>
+      </c>
+      <c r="G39" s="14">
+        <v>0</v>
+      </c>
+      <c r="H39" s="14">
+        <v>45</v>
+      </c>
+      <c r="I39" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J39" s="15" t="str">
+        <v>950</v>
+      </c>
+      <c r="J39" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K39" s="16"/>
-      <c r="L39" s="16"/>
-      <c r="M39" s="16"/>
-      <c r="N39" s="17"/>
+        <v>490</v>
+      </c>
+      <c r="K39" s="16" t="s">
+        <v>59</v>
+      </c>
+      <c r="L39" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="M39" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="N39" s="17" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="40" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A40" s="13"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14"/>
-      <c r="D40" s="14"/>
-      <c r="E40" s="14"/>
-      <c r="F40" s="14"/>
-      <c r="G40" s="14"/>
-      <c r="H40" s="14"/>
-      <c r="I40" s="15" t="str">
+      <c r="A40" s="13">
+        <v>46294</v>
+      </c>
+      <c r="B40" s="14">
+        <v>600</v>
+      </c>
+      <c r="C40" s="14">
+        <v>5</v>
+      </c>
+      <c r="D40" s="14">
+        <v>200</v>
+      </c>
+      <c r="E40" s="14">
+        <v>230</v>
+      </c>
+      <c r="F40" s="14">
+        <v>0</v>
+      </c>
+      <c r="G40" s="14">
+        <v>0</v>
+      </c>
+      <c r="H40" s="14">
+        <v>30</v>
+      </c>
+      <c r="I40" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J40" s="15" t="str">
+        <v>1065</v>
+      </c>
+      <c r="J40" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K40" s="16"/>
-      <c r="L40" s="16"/>
-      <c r="M40" s="16"/>
-      <c r="N40" s="17"/>
+        <v>375</v>
+      </c>
+      <c r="K40" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="L40" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M40" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N40" s="17" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="41" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A41" s="13"/>

</xml_diff>

<commit_message>
main10 and 11 oct
</commit_message>
<xml_diff>
--- a/12604997.xlsx
+++ b/12604997.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98B5B45D-8312-402A-BD39-2EAD12A0BACB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E579CFB-4816-40AC-90E2-2B299DC69B0D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="241" uniqueCount="86">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -3142,48 +3142,96 @@
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="13"/>
-      <c r="B51" s="14"/>
-      <c r="C51" s="14"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="14"/>
-      <c r="G51" s="14"/>
-      <c r="H51" s="14"/>
-      <c r="I51" s="15" t="str">
+      <c r="A51" s="13">
+        <v>46305</v>
+      </c>
+      <c r="B51" s="14">
+        <v>560</v>
+      </c>
+      <c r="C51" s="14">
+        <v>45</v>
+      </c>
+      <c r="D51" s="14">
+        <v>200</v>
+      </c>
+      <c r="E51" s="14">
+        <v>45</v>
+      </c>
+      <c r="F51" s="14">
+        <v>0</v>
+      </c>
+      <c r="G51" s="14">
+        <v>0</v>
+      </c>
+      <c r="H51" s="14">
+        <v>65</v>
+      </c>
+      <c r="I51" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="15" t="str">
+        <v>915</v>
+      </c>
+      <c r="J51" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="16"/>
-      <c r="L51" s="16"/>
-      <c r="M51" s="16"/>
-      <c r="N51" s="17"/>
+        <v>525</v>
+      </c>
+      <c r="K51" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="L51" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M51" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N51" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="13"/>
-      <c r="B52" s="14"/>
-      <c r="C52" s="14"/>
-      <c r="D52" s="14"/>
-      <c r="E52" s="14"/>
-      <c r="F52" s="14"/>
-      <c r="G52" s="14"/>
-      <c r="H52" s="14"/>
-      <c r="I52" s="15" t="str">
+      <c r="A52" s="13">
+        <v>46306</v>
+      </c>
+      <c r="B52" s="14">
+        <v>580</v>
+      </c>
+      <c r="C52" s="14">
+        <v>55</v>
+      </c>
+      <c r="D52" s="14">
+        <v>250</v>
+      </c>
+      <c r="E52" s="14">
+        <v>55</v>
+      </c>
+      <c r="F52" s="14">
+        <v>0</v>
+      </c>
+      <c r="G52" s="14">
+        <v>0</v>
+      </c>
+      <c r="H52" s="14">
+        <v>75</v>
+      </c>
+      <c r="I52" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="15" t="str">
+        <v>1015</v>
+      </c>
+      <c r="J52" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="16"/>
-      <c r="L52" s="16"/>
-      <c r="M52" s="16"/>
-      <c r="N52" s="17"/>
+        <v>425</v>
+      </c>
+      <c r="K52" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="L52" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="M52" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="N52" s="17" t="s">
+        <v>58</v>
+      </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
       <c r="A53" s="13"/>

</xml_diff>